<commit_message>
update HForms XLS xml_node_name to repeat_xml_node
</commit_message>
<xml_diff>
--- a/app/src/main/res/raw/change_head_form.xlsx
+++ b/app/src/main/res/raw/change_head_form.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27645" windowHeight="11970" tabRatio="500" activeTab="1"/>
+    <workbookView windowWidth="22620" windowHeight="12090" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="columns" sheetId="1" r:id="rId1"/>
@@ -784,7 +784,7 @@
     <t>repeat_name</t>
   </si>
   <si>
-    <t>xml_node_name</t>
+    <t>repeat_xml_node</t>
   </si>
   <si>
     <t>rawChangeHead</t>
@@ -810,10 +810,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="28">
     <font>
@@ -862,16 +862,40 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="0"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -885,13 +909,58 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -912,17 +981,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -936,71 +996,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1048,7 +1048,79 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1060,31 +1132,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1096,19 +1204,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1120,115 +1222,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1336,6 +1336,24 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -1351,11 +1369,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1379,172 +1403,148 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="34" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">

</xml_diff>

<commit_message>
Update HForms - removing not needed repeat_count variable
</commit_message>
<xml_diff>
--- a/app/src/main/res/raw/change_head_form.xlsx
+++ b/app/src/main/res/raw/change_head_form.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22620" windowHeight="12090" tabRatio="500" activeTab="2"/>
+    <workbookView windowWidth="22770" windowHeight="12315" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="columns" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="250">
   <si>
     <t>group</t>
   </si>
@@ -269,9 +269,6 @@
   </si>
   <si>
     <t>start repeat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$household_residents </t>
   </si>
   <si>
     <t>5. Relationships of Members with the new Head of Household</t>
@@ -810,10 +807,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="28">
     <font>
@@ -853,6 +850,58 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -861,8 +910,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -885,82 +935,15 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -981,8 +964,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -996,9 +980,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1054,7 +1051,73 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1066,7 +1129,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1078,127 +1195,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1210,25 +1213,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1306,32 +1303,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="double">
-        <color rgb="FF3F3F3F"/>
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1384,6 +1360,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -1395,159 +1386,165 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2332,20 +2329,18 @@
         <v>72</v>
       </c>
       <c r="F11" s="37"/>
-      <c r="G11" s="37" t="s">
+      <c r="G11" s="37"/>
+      <c r="H11" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="H11" s="38" t="s">
+      <c r="I11" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="I11" s="38" t="s">
+      <c r="J11" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="J11" s="45" t="s">
+      <c r="K11" s="46" t="s">
         <v>76</v>
-      </c>
-      <c r="K11" s="46" t="s">
-        <v>77</v>
       </c>
       <c r="L11" s="46"/>
       <c r="M11" s="46"/>
@@ -2358,25 +2353,25 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" t="s">
         <v>78</v>
-      </c>
-      <c r="D12" t="s">
-        <v>79</v>
       </c>
       <c r="E12" t="s">
         <v>20</v>
       </c>
       <c r="H12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I12" t="s">
         <v>80</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="K12" s="44" t="s">
         <v>82</v>
-      </c>
-      <c r="K12" s="44" t="s">
-        <v>83</v>
       </c>
       <c r="L12" s="44"/>
       <c r="M12" s="44"/>
@@ -2389,25 +2384,25 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
         <v>20</v>
       </c>
       <c r="H13" t="s">
+        <v>84</v>
+      </c>
+      <c r="I13" t="s">
         <v>85</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="K13" s="44" t="s">
         <v>87</v>
-      </c>
-      <c r="K13" s="44" t="s">
-        <v>88</v>
       </c>
       <c r="L13" s="44"/>
       <c r="M13" s="44"/>
@@ -2421,25 +2416,25 @@
     <row r="14" spans="1:14">
       <c r="A14" s="1"/>
       <c r="D14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E14" t="s">
         <v>89</v>
-      </c>
-      <c r="E14" t="s">
-        <v>90</v>
       </c>
       <c r="F14" s="30" t="s">
         <v>71</v>
       </c>
       <c r="H14" t="s">
+        <v>90</v>
+      </c>
+      <c r="I14" t="s">
         <v>91</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="K14" s="44" t="s">
         <v>93</v>
-      </c>
-      <c r="K14" s="44" t="s">
-        <v>94</v>
       </c>
       <c r="L14" s="44"/>
       <c r="M14" s="44"/>
@@ -2455,7 +2450,7 @@
         <v>71</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F15" s="39"/>
       <c r="G15" s="39"/>
@@ -2472,27 +2467,27 @@
     </row>
     <row r="16" s="27" customFormat="1" spans="1:15">
       <c r="A16" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="E16" s="27" t="s">
         <v>97</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>98</v>
       </c>
       <c r="F16" s="40"/>
       <c r="G16" s="40"/>
       <c r="H16" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="I16" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="I16" s="27" t="s">
+      <c r="J16" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="K16" s="47" t="s">
         <v>101</v>
-      </c>
-      <c r="K16" s="47" t="s">
-        <v>102</v>
       </c>
       <c r="L16" s="47"/>
       <c r="M16" s="47"/>
@@ -2505,27 +2500,27 @@
     </row>
     <row r="17" s="28" customFormat="1" spans="1:15">
       <c r="A17" s="35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D17" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="E17" s="28" t="s">
         <v>103</v>
-      </c>
-      <c r="E17" s="28" t="s">
-        <v>104</v>
       </c>
       <c r="F17" s="41"/>
       <c r="G17" s="41"/>
       <c r="H17" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="I17" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="I17" s="28" t="s">
+      <c r="J17" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="K17" s="48" t="s">
         <v>107</v>
-      </c>
-      <c r="K17" s="48" t="s">
-        <v>108</v>
       </c>
       <c r="L17" s="48"/>
       <c r="M17" s="48"/>
@@ -2538,25 +2533,25 @@
     </row>
     <row r="18" s="28" customFormat="1" spans="1:18">
       <c r="A18" s="35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D18" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="H18" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="I18" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="K18" s="48" t="s">
         <v>111</v>
-      </c>
-      <c r="I18" s="28" t="s">
-        <v>111</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="K18" s="48" t="s">
-        <v>112</v>
       </c>
       <c r="L18" s="48"/>
       <c r="M18" s="48"/>
@@ -2569,25 +2564,25 @@
     </row>
     <row r="19" s="28" customFormat="1" spans="1:18">
       <c r="A19" s="35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E19" s="28" t="s">
         <v>20</v>
       </c>
       <c r="H19" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="I19" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K19" s="48" t="s">
         <v>114</v>
-      </c>
-      <c r="I19" s="28" t="s">
-        <v>114</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="K19" s="48" t="s">
-        <v>115</v>
       </c>
       <c r="L19" s="48"/>
       <c r="M19" s="48"/>
@@ -2600,25 +2595,25 @@
     </row>
     <row r="20" s="28" customFormat="1" spans="1:18">
       <c r="A20" s="35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E20" s="28" t="s">
         <v>20</v>
       </c>
       <c r="H20" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="I20" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K20" s="48" t="s">
         <v>117</v>
-      </c>
-      <c r="I20" s="28" t="s">
-        <v>117</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="K20" s="48" t="s">
-        <v>118</v>
       </c>
       <c r="L20" s="48"/>
       <c r="M20" s="48"/>
@@ -2631,10 +2626,10 @@
     </row>
     <row r="21" s="29" customFormat="1" spans="1:15">
       <c r="A21" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E21" s="29" t="s">
         <v>20</v>
@@ -2642,16 +2637,16 @@
       <c r="F21" s="42"/>
       <c r="G21" s="42"/>
       <c r="H21" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="I21" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="I21" s="29" t="s">
+      <c r="J21" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="K21" s="49" t="s">
         <v>122</v>
-      </c>
-      <c r="K21" s="49" t="s">
-        <v>123</v>
       </c>
       <c r="L21" s="49"/>
       <c r="M21" s="49"/>
@@ -2745,7 +2740,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
@@ -2765,85 +2760,85 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B2" s="1" t="b">
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" t="s">
         <v>126</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="F2" s="20" t="s">
         <v>128</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>129</v>
       </c>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B3" s="1" t="b">
         <v>0</v>
       </c>
       <c r="C3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" t="s">
         <v>130</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="F3" s="20" t="s">
         <v>132</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>133</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="F4" s="22" t="s">
         <v>138</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>139</v>
       </c>
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="F5" s="22" t="s">
         <v>143</v>
-      </c>
-      <c r="F5" s="22" t="s">
-        <v>144</v>
       </c>
       <c r="G5" s="5"/>
     </row>
@@ -2852,22 +2847,22 @@
         <v>71</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="F6" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="G6" s="24" t="s">
         <v>149</v>
-      </c>
-      <c r="G6" s="24" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2875,19 +2870,19 @@
         <v>71</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="F7" s="20" t="s">
         <v>154</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2895,19 +2890,19 @@
         <v>71</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="D8" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="E8" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="F8" s="20" t="s">
         <v>159</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2915,19 +2910,19 @@
         <v>71</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="F9" s="20" t="s">
         <v>164</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2935,19 +2930,19 @@
         <v>71</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="E10" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="F10" s="20" t="s">
         <v>169</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2955,19 +2950,19 @@
         <v>71</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="D11" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="E11" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="F11" s="20" t="s">
         <v>174</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2975,19 +2970,19 @@
         <v>71</v>
       </c>
       <c r="B12" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="D12" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="F12" s="20" t="s">
         <v>179</v>
-      </c>
-      <c r="F12" s="20" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2995,19 +2990,19 @@
         <v>71</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="E13" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="F13" s="20" t="s">
         <v>184</v>
-      </c>
-      <c r="F13" s="20" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -3015,39 +3010,39 @@
         <v>71</v>
       </c>
       <c r="B14" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="D14" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="E14" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="F14" s="20" t="s">
         <v>189</v>
-      </c>
-      <c r="F14" s="20" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" t="s">
         <v>192</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>193</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="F15" s="20" t="s">
         <v>195</v>
-      </c>
-      <c r="F15" s="20" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="16" s="4" customFormat="1" spans="1:6">
@@ -3055,19 +3050,19 @@
         <v>60</v>
       </c>
       <c r="B16" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C16" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="D16" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="F16" s="26" t="s">
         <v>200</v>
-      </c>
-      <c r="F16" s="26" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="17" s="4" customFormat="1" spans="1:6">
@@ -3075,19 +3070,19 @@
         <v>60</v>
       </c>
       <c r="B17" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="C17" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="D17" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="F17" s="26" t="s">
         <v>205</v>
-      </c>
-      <c r="F17" s="26" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="18" s="4" customFormat="1" spans="1:6">
@@ -3095,19 +3090,19 @@
         <v>60</v>
       </c>
       <c r="B18" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C18" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="D18" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="F18" s="26" t="s">
         <v>210</v>
-      </c>
-      <c r="F18" s="26" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="19" s="4" customFormat="1" spans="1:6">
@@ -3115,19 +3110,19 @@
         <v>60</v>
       </c>
       <c r="B19" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="C19" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="D19" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="F19" s="26" t="s">
         <v>215</v>
-      </c>
-      <c r="F19" s="26" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="20" s="4" customFormat="1" spans="1:6">
@@ -3135,19 +3130,19 @@
         <v>60</v>
       </c>
       <c r="B20" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="C20" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="D20" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="E20" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="F20" s="26" t="s">
         <v>220</v>
-      </c>
-      <c r="F20" s="26" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="21" s="4" customFormat="1" spans="1:6">
@@ -3155,19 +3150,19 @@
         <v>60</v>
       </c>
       <c r="B21" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="D21" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="E21" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="F21" s="26" t="s">
         <v>225</v>
-      </c>
-      <c r="F21" s="26" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="22" s="4" customFormat="1" spans="1:6">
@@ -3175,19 +3170,19 @@
         <v>60</v>
       </c>
       <c r="B22" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="C22" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="D22" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="F22" s="26" t="s">
         <v>230</v>
-      </c>
-      <c r="F22" s="26" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="23" s="4" customFormat="1" spans="1:6">
@@ -3195,19 +3190,19 @@
         <v>60</v>
       </c>
       <c r="B23" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="C23" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="D23" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="F23" s="26" t="s">
         <v>235</v>
-      </c>
-      <c r="F23" s="26" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -3396,45 +3391,45 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" t="s">
         <v>238</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" t="s">
         <v>240</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>241</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>243</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B2" t="s">
         <v>245</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>246</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>249</v>
       </c>
       <c r="F2" s="1">
         <v>1</v>
@@ -3443,7 +3438,7 @@
         <v>71</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- Add support for "$external" constant on HForms repeat_count to specify that the repeat group objects will be externally loaded - Add constant variable "$external" to HForms repeat_count column for forms that are loading repeat objects externally   - affected forms: change_head_form, death_form, pregnancy_outcome_form, pregnancy_visit_form
</commit_message>
<xml_diff>
--- a/app/src/main/res/raw/change_head_form.xlsx
+++ b/app/src/main/res/raw/change_head_form.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22770" windowHeight="12315" tabRatio="500"/>
+    <workbookView windowWidth="27795" windowHeight="12315" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="columns" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="251">
   <si>
     <t>group</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t>start repeat</t>
+  </si>
+  <si>
+    <t>$external</t>
   </si>
   <si>
     <t>5. Relationships of Members with the new Head of Household</t>
@@ -808,8 +811,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="28">
@@ -850,46 +853,9 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -898,13 +864,20 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -912,6 +885,36 @@
     <font>
       <b/>
       <sz val="13"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -926,8 +929,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -935,15 +953,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -951,22 +961,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -981,21 +975,30 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF3F3F76"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1045,7 +1048,163 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1057,169 +1216,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1303,11 +1306,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1317,6 +1326,36 @@
       <top/>
       <bottom style="medium">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1345,32 +1384,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1385,166 +1403,151 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1614,6 +1617,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1624,7 +1628,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1634,13 +1637,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1654,8 +1654,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -1981,8 +1982,8 @@
     <col min="3" max="3" width="14.1809523809524" customWidth="1"/>
     <col min="4" max="4" width="20.1809523809524" customWidth="1"/>
     <col min="5" max="5" width="11.7238095238095" customWidth="1"/>
-    <col min="6" max="6" width="12" style="30" customWidth="1"/>
-    <col min="7" max="7" width="20" style="30" customWidth="1"/>
+    <col min="6" max="6" width="12" style="31" customWidth="1"/>
+    <col min="7" max="7" width="20" style="31" customWidth="1"/>
     <col min="8" max="8" width="51.5428571428571" customWidth="1"/>
     <col min="9" max="10" width="55" customWidth="1"/>
     <col min="11" max="11" width="41.6666666666667" customWidth="1"/>
@@ -2008,10 +2009,10 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="30" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="30" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -2038,7 +2039,7 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="30" t="s">
+      <c r="P1" s="31" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
@@ -2069,7 +2070,7 @@
       <c r="J2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="43" t="s">
+      <c r="K2" s="42" t="s">
         <v>24</v>
       </c>
       <c r="L2" s="1"/>
@@ -2080,7 +2081,7 @@
       <c r="O2" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P2" s="30"/>
+      <c r="P2" s="31"/>
     </row>
     <row r="3" spans="1:16">
       <c r="A3" s="1" t="s">
@@ -2103,7 +2104,7 @@
       <c r="J3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="43" t="s">
+      <c r="K3" s="42" t="s">
         <v>29</v>
       </c>
       <c r="L3" s="1"/>
@@ -2114,7 +2115,7 @@
       <c r="O3" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="P3" s="30"/>
+      <c r="P3" s="31"/>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="1" t="s">
@@ -2135,11 +2136,11 @@
       <c r="J4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="K4" s="44" t="s">
+      <c r="K4" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="44"/>
-      <c r="M4" s="44"/>
+      <c r="L4" s="43"/>
+      <c r="M4" s="43"/>
       <c r="O4" t="b">
         <v>1</v>
       </c>
@@ -2163,11 +2164,11 @@
       <c r="J5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="K5" s="44" t="s">
+      <c r="K5" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="L5" s="44"/>
-      <c r="M5" s="44"/>
+      <c r="L5" s="43"/>
+      <c r="M5" s="43"/>
       <c r="O5" t="b">
         <v>1</v>
       </c>
@@ -2191,11 +2192,11 @@
       <c r="J6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="K6" s="44" t="s">
+      <c r="K6" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="L6" s="44"/>
-      <c r="M6" s="44"/>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
       <c r="N6" t="b">
         <v>1</v>
       </c>
@@ -2222,11 +2223,11 @@
       <c r="J7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="K7" s="44" t="s">
+      <c r="K7" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="L7" s="44"/>
-      <c r="M7" s="44"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
       <c r="N7" t="b">
         <v>1</v>
       </c>
@@ -2251,11 +2252,11 @@
       <c r="J8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="K8" s="44" t="s">
+      <c r="K8" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="44"/>
-      <c r="M8" s="44"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
       <c r="N8" t="b">
         <v>1</v>
       </c>
@@ -2268,7 +2269,7 @@
       <c r="E9" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="30" t="s">
+      <c r="F9" s="31" t="s">
         <v>60</v>
       </c>
       <c r="H9" t="s">
@@ -2280,11 +2281,11 @@
       <c r="J9" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="K9" s="44" t="s">
+      <c r="K9" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="L9" s="44"/>
-      <c r="M9" s="44"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="43"/>
       <c r="N9" t="b">
         <v>1</v>
       </c>
@@ -2306,11 +2307,11 @@
       <c r="J10" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="K10" s="44" t="s">
+      <c r="K10" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
+      <c r="L10" s="43"/>
+      <c r="M10" s="43"/>
       <c r="N10" t="b">
         <v>1</v>
       </c>
@@ -2318,10 +2319,10 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
-      <c r="A11" s="31"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
+    <row r="11" s="27" customFormat="1" spans="1:17">
+      <c r="A11" s="32"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
       <c r="D11" s="33" t="s">
         <v>71</v>
       </c>
@@ -2329,18 +2330,20 @@
         <v>72</v>
       </c>
       <c r="F11" s="37"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="38" t="s">
+      <c r="G11" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="I11" s="38" t="s">
+      <c r="H11" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="J11" s="45" t="s">
+      <c r="I11" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="K11" s="46" t="s">
+      <c r="J11" s="44" t="s">
         <v>76</v>
+      </c>
+      <c r="K11" s="45" t="s">
+        <v>77</v>
       </c>
       <c r="L11" s="46"/>
       <c r="M11" s="46"/>
@@ -2353,28 +2356,28 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E12" t="s">
         <v>20</v>
       </c>
       <c r="H12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="K12" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="L12" s="44"/>
-      <c r="M12" s="44"/>
+      <c r="K12" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="L12" s="43"/>
+      <c r="M12" s="43"/>
       <c r="N12" t="b">
         <v>1</v>
       </c>
@@ -2384,28 +2387,28 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E13" t="s">
         <v>20</v>
       </c>
       <c r="H13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="K13" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="L13" s="44"/>
-      <c r="M13" s="44"/>
+      <c r="K13" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="L13" s="43"/>
+      <c r="M13" s="43"/>
       <c r="N13" t="b">
         <v>1</v>
       </c>
@@ -2416,44 +2419,44 @@
     <row r="14" spans="1:14">
       <c r="A14" s="1"/>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>89</v>
-      </c>
-      <c r="F14" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="F14" s="31" t="s">
         <v>71</v>
       </c>
       <c r="H14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="K14" s="44" t="s">
         <v>93</v>
       </c>
-      <c r="L14" s="44"/>
-      <c r="M14" s="44"/>
+      <c r="K14" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="L14" s="43"/>
+      <c r="M14" s="43"/>
       <c r="N14" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
-      <c r="A15" s="31"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
+    <row r="15" s="27" customFormat="1" spans="1:17">
+      <c r="A15" s="32"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
       <c r="D15" s="33" t="s">
         <v>71</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>94</v>
-      </c>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
+        <v>95</v>
+      </c>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
       <c r="H15" s="38"/>
       <c r="I15" s="38"/>
       <c r="J15" s="38"/>
@@ -2465,221 +2468,221 @@
       <c r="P15" s="38"/>
       <c r="Q15" s="38"/>
     </row>
-    <row r="16" s="27" customFormat="1" spans="1:15">
+    <row r="16" s="28" customFormat="1" spans="1:15">
       <c r="A16" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="D16" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="D16" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="27" t="s">
+      <c r="E16" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="I16" s="27" t="s">
+      <c r="F16" s="39"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="28" t="s">
         <v>99</v>
       </c>
+      <c r="I16" s="28" t="s">
+        <v>100</v>
+      </c>
       <c r="J16" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K16" s="47" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L16" s="47"/>
       <c r="M16" s="47"/>
-      <c r="N16" s="27" t="b">
+      <c r="N16" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="O16" s="27" t="b">
+      <c r="O16" s="28" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" s="28" customFormat="1" spans="1:15">
+    <row r="17" s="29" customFormat="1" spans="1:15">
       <c r="A17" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>102</v>
-      </c>
-      <c r="E17" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="F17" s="41"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="28" t="s">
+      <c r="E17" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="I17" s="28" t="s">
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="29" t="s">
         <v>105</v>
       </c>
+      <c r="I17" s="29" t="s">
+        <v>106</v>
+      </c>
       <c r="J17" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K17" s="48" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L17" s="48"/>
       <c r="M17" s="48"/>
-      <c r="N17" s="28" t="b">
+      <c r="N17" s="29" t="b">
         <v>1</v>
       </c>
-      <c r="O17" s="28" t="b">
+      <c r="O17" s="29" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" s="28" customFormat="1" spans="1:18">
+    <row r="18" s="29" customFormat="1" spans="1:18">
       <c r="A18" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="E18" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" s="29" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="E18" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="I18" s="28" t="s">
-        <v>110</v>
+      <c r="H18" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="I18" s="29" t="s">
+        <v>111</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K18" s="48" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L18" s="48"/>
       <c r="M18" s="48"/>
-      <c r="O18" s="28" t="b">
+      <c r="O18" s="29" t="b">
         <v>1</v>
       </c>
-      <c r="R18" s="28" t="b">
+      <c r="R18" s="29" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" s="28" customFormat="1" spans="1:18">
+    <row r="19" s="29" customFormat="1" spans="1:18">
       <c r="A19" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="E19" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="E19" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="H19" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="I19" s="28" t="s">
-        <v>113</v>
+      <c r="H19" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="I19" s="29" t="s">
+        <v>114</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K19" s="48" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L19" s="48"/>
       <c r="M19" s="48"/>
-      <c r="O19" s="28" t="b">
+      <c r="O19" s="29" t="b">
         <v>1</v>
       </c>
-      <c r="R19" s="28" t="b">
+      <c r="R19" s="29" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="20" s="28" customFormat="1" spans="1:18">
+    <row r="20" s="29" customFormat="1" spans="1:18">
       <c r="A20" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="E20" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="H20" s="28" t="s">
-        <v>116</v>
-      </c>
-      <c r="I20" s="28" t="s">
-        <v>116</v>
+      <c r="H20" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" s="29" t="s">
+        <v>117</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K20" s="48" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L20" s="48"/>
       <c r="M20" s="48"/>
-      <c r="O20" s="28" t="b">
+      <c r="O20" s="29" t="b">
         <v>1</v>
       </c>
-      <c r="R20" s="28" t="b">
+      <c r="R20" s="29" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="21" s="29" customFormat="1" spans="1:15">
+    <row r="21" s="30" customFormat="1" spans="1:15">
       <c r="A21" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="E21" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="I21" s="29" t="s">
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="30" t="s">
         <v>120</v>
       </c>
+      <c r="I21" s="30" t="s">
+        <v>121</v>
+      </c>
       <c r="J21" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K21" s="49" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="L21" s="49"/>
       <c r="M21" s="49"/>
-      <c r="N21" s="29" t="b">
+      <c r="N21" s="30" t="b">
         <v>1</v>
       </c>
-      <c r="O21" s="29" t="b">
+      <c r="O21" s="30" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="1"/>
-      <c r="K22" s="44"/>
-      <c r="L22" s="44"/>
-      <c r="M22" s="44"/>
+      <c r="K22" s="43"/>
+      <c r="L22" s="43"/>
+      <c r="M22" s="43"/>
     </row>
     <row r="23" spans="1:13">
       <c r="A23" s="1"/>
-      <c r="K23" s="44"/>
-      <c r="L23" s="44"/>
-      <c r="M23" s="44"/>
+      <c r="K23" s="43"/>
+      <c r="L23" s="43"/>
+      <c r="M23" s="43"/>
     </row>
     <row r="24" spans="1:13">
       <c r="A24" s="1"/>
-      <c r="K24" s="44"/>
-      <c r="L24" s="44"/>
-      <c r="M24" s="44"/>
+      <c r="K24" s="43"/>
+      <c r="L24" s="43"/>
+      <c r="M24" s="43"/>
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="1"/>
-      <c r="K25" s="44"/>
-      <c r="L25" s="44"/>
-      <c r="M25" s="44"/>
+      <c r="K25" s="43"/>
+      <c r="L25" s="43"/>
+      <c r="M25" s="43"/>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="1"/>
@@ -2740,7 +2743,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
@@ -2760,85 +2763,85 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B2" s="1" t="b">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B3" s="1" t="b">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G5" s="5"/>
     </row>
@@ -2847,22 +2850,22 @@
         <v>71</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2870,19 +2873,19 @@
         <v>71</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2890,19 +2893,19 @@
         <v>71</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2910,19 +2913,19 @@
         <v>71</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2930,19 +2933,19 @@
         <v>71</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2950,19 +2953,19 @@
         <v>71</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2970,19 +2973,19 @@
         <v>71</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E12" s="25" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2990,19 +2993,19 @@
         <v>71</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -3010,39 +3013,39 @@
         <v>71</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E14" s="25" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" s="4" customFormat="1" spans="1:6">
@@ -3050,19 +3053,19 @@
         <v>60</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" s="4" customFormat="1" spans="1:6">
@@ -3070,19 +3073,19 @@
         <v>60</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" s="4" customFormat="1" spans="1:6">
@@ -3090,19 +3093,19 @@
         <v>60</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" s="4" customFormat="1" spans="1:6">
@@ -3110,19 +3113,19 @@
         <v>60</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F19" s="26" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="20" s="4" customFormat="1" spans="1:6">
@@ -3130,19 +3133,19 @@
         <v>60</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="21" s="4" customFormat="1" spans="1:6">
@@ -3150,19 +3153,19 @@
         <v>60</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="22" s="4" customFormat="1" spans="1:6">
@@ -3170,19 +3173,19 @@
         <v>60</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F22" s="26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="23" s="4" customFormat="1" spans="1:6">
@@ -3190,19 +3193,19 @@
         <v>60</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F23" s="26" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -3391,45 +3394,45 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F2" s="1">
         <v>1</v>
@@ -3438,7 +3441,7 @@
         <v>71</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>